<commit_message>
Release web 1.8.0 R11: catalog slider, quantity rules and customer checkout
</commit_message>
<xml_diff>
--- a/actualizaciones/1.8.0/web/assets/machote-productos.xlsx
+++ b/actualizaciones/1.8.0/web/assets/machote-productos.xlsx
@@ -568,7 +568,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opcional. unidad por defecto; ejemplo kg o pieza. Hasta 40 caracteres.</t>
+          <t xml:space="preserve">Opcional. unidad por defecto: sólo enteros. Para granel indica kg, g, litros o metros. Hasta 40 caracteres.</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opcional. 1 por defecto. Mayor que 0 y acorde a decimales.</t>
+          <t xml:space="preserve">Unidad: 1. Granel: mayor que 0 y acorde a decimales; ejemplo 0.25.</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opcional. 1 por defecto. Mayor que 0 y acorde a decimales.</t>
+          <t xml:space="preserve">Unidad: 1. Granel: mayor que 0 y acorde a decimales; ejemplo 0.25.</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opcional. 0 por defecto. Entero entre 0 y 3 para venta por cantidad.</t>
+          <t xml:space="preserve">Unidad: 0. Granel: 1 a 3; si dejas la configuración vacía, se propone precisión 3.</t>
         </is>
       </c>
     </row>

</xml_diff>